<commit_message>
feat: update books table from Excel — 532 books (+5 new)
</commit_message>
<xml_diff>
--- a/Книги.xlsx
+++ b/Книги.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dmitrypotekhin/Downloads/dmpotekhin.github.io/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02B342AC-36A9-8D4A-BEB8-D78346198B29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81C502F7-181D-2E43-A964-0355164D7B3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="16000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1583" uniqueCount="861">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1595" uniqueCount="868">
   <si>
     <t>Борис Акунин</t>
   </si>
@@ -2607,6 +2607,27 @@
   </si>
   <si>
     <t>Путешествие в Сиам</t>
+  </si>
+  <si>
+    <t>Ли Бао</t>
+  </si>
+  <si>
+    <t>Китайская Культурная Революция</t>
+  </si>
+  <si>
+    <t>Путешествие на Новую Гвинею</t>
+  </si>
+  <si>
+    <t>Николай Миклохо-Маклай</t>
+  </si>
+  <si>
+    <t>Собака на сене</t>
+  </si>
+  <si>
+    <t>Лопе де Вега</t>
+  </si>
+  <si>
+    <t>100 млн модель продаж</t>
   </si>
 </sst>
 </file>
@@ -2909,7 +2930,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:U529"/>
+  <dimension ref="A1:U533"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -9539,8 +9560,53 @@
         <v>169</v>
       </c>
     </row>
+    <row r="530" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A530" s="5" t="s">
+        <v>861</v>
+      </c>
+      <c r="B530" s="5" t="s">
+        <v>862</v>
+      </c>
+      <c r="C530" s="5" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="531" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A531" s="5" t="s">
+        <v>864</v>
+      </c>
+      <c r="B531" s="5" t="s">
+        <v>863</v>
+      </c>
+      <c r="C531" s="5" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="532" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A532" s="5" t="s">
+        <v>866</v>
+      </c>
+      <c r="B532" s="5" t="s">
+        <v>865</v>
+      </c>
+      <c r="C532" s="5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="533" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A533" s="5" t="s">
+        <v>850</v>
+      </c>
+      <c r="B533" s="5" t="s">
+        <v>867</v>
+      </c>
+      <c r="C533" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C508" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update books from Excel — 533 books (+1: 100 млн модель Лиды)
</commit_message>
<xml_diff>
--- a/Книги.xlsx
+++ b/Книги.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dmitrypotekhin/Downloads/dmpotekhin.github.io/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81C502F7-181D-2E43-A964-0355164D7B3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B34B3BF-DAA1-C342-8367-4C0353E2D633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="16000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1595" uniqueCount="868">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1598" uniqueCount="869">
   <si>
     <t>Борис Акунин</t>
   </si>
@@ -2628,6 +2628,9 @@
   </si>
   <si>
     <t>100 млн модель продаж</t>
+  </si>
+  <si>
+    <t>100 млн модель Лиды</t>
   </si>
 </sst>
 </file>
@@ -2930,7 +2933,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:U533"/>
+  <dimension ref="A1:U534"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -9604,6 +9607,17 @@
         <v>70</v>
       </c>
     </row>
+    <row r="534" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A534" s="5" t="s">
+        <v>850</v>
+      </c>
+      <c r="B534" s="5" t="s">
+        <v>868</v>
+      </c>
+      <c r="C534" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C508" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: update books from Excel — 535 books (+44 new notes)
</commit_message>
<xml_diff>
--- a/Книги.xlsx
+++ b/Книги.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dmitrypotekhin/Downloads/dmpotekhin.github.io/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B34B3BF-DAA1-C342-8367-4C0353E2D633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61823D8C-1C31-F046-8BAE-603A4BD136D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="16000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1598" uniqueCount="869">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1604" uniqueCount="873">
   <si>
     <t>Борис Акунин</t>
   </si>
@@ -2631,6 +2631,18 @@
   </si>
   <si>
     <t>100 млн модель Лиды</t>
+  </si>
+  <si>
+    <t>Искусство видеть</t>
+  </si>
+  <si>
+    <t>Джон Бергер</t>
+  </si>
+  <si>
+    <t>Анастасия Постригай</t>
+  </si>
+  <si>
+    <t>Влюбиться в исскуство</t>
   </si>
 </sst>
 </file>
@@ -2933,7 +2945,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:U534"/>
+  <dimension ref="A1:U536"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -9618,6 +9630,28 @@
         <v>70</v>
       </c>
     </row>
+    <row r="535" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A535" s="5" t="s">
+        <v>870</v>
+      </c>
+      <c r="B535" s="5" t="s">
+        <v>869</v>
+      </c>
+      <c r="C535" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="536" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A536" s="5" t="s">
+        <v>871</v>
+      </c>
+      <c r="B536" s="5" t="s">
+        <v>872</v>
+      </c>
+      <c r="C536" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C508" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>